<commit_message>
updated home related test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/InternalContact_Field_Values.xlsx
+++ b/src/main/resources/InternalContact_Field_Values.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22624"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A7DBF1-D7B9-4BE3-A1C5-586D9B6A6461}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51A98269-0960-4232-BF96-1D8AF30AF904}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="3" r:id="rId1"/>
@@ -123,10 +123,10 @@
     <t>SterlingREI</t>
   </si>
   <si>
-    <t>Automation Runtime</t>
-  </si>
-  <si>
     <t>Contact</t>
+  </si>
+  <si>
+    <t>Automation Runtime Contact</t>
   </si>
 </sst>
 </file>
@@ -465,14 +465,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D795F61-CC1F-4314-B1D8-0852B981BA18}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="23.109375" customWidth="1"/>
-    <col min="2" max="2" width="21.44140625" customWidth="1"/>
-    <col min="3" max="3" width="37.21875" customWidth="1"/>
+    <col min="1" max="1" width="23.07421875" customWidth="1"/>
+    <col min="2" max="2" width="21.4609375" customWidth="1"/>
+    <col min="3" max="3" width="37.23046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -483,7 +483,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -491,10 +491,10 @@
         <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -502,10 +502,10 @@
         <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -516,7 +516,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -527,7 +527,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -538,7 +538,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -549,7 +549,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -560,7 +560,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -571,7 +571,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -582,7 +582,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -593,7 +593,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -604,7 +604,7 @@
         <v>20171</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -627,13 +627,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA6F275D-7657-4500-825C-5F565736E8FE}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.23046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -644,7 +644,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -655,7 +655,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -666,7 +666,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -689,14 +689,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F187A448-1415-4E32-A6B0-57F6ABB88CB8}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.765625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -707,7 +707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Updated as per modification in test case
</commit_message>
<xml_diff>
--- a/src/main/resources/InternalContact_Field_Values.xlsx
+++ b/src/main/resources/InternalContact_Field_Values.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EFC048E-D4BA-4D56-872F-9A72F306B463}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CD56785-EA83-4CC4-820F-3C72DC42B7D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="34">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -54,33 +54,15 @@
     <t>PREG</t>
   </si>
   <si>
-    <t>AccountId</t>
-  </si>
-  <si>
-    <t>FirstName</t>
-  </si>
-  <si>
-    <t>LastName</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
     <t>None</t>
   </si>
   <si>
     <t>Phone</t>
   </si>
   <si>
-    <t>Salutation</t>
-  </si>
-  <si>
     <t>Ms.</t>
   </si>
   <si>
-    <t>Primary</t>
-  </si>
-  <si>
     <t>(701)-346-5555</t>
   </si>
   <si>
@@ -123,17 +105,32 @@
     <t>fieldMailingCountry</t>
   </si>
   <si>
-    <t>fieldUserRole__c</t>
-  </si>
-  <si>
     <t>VA</t>
+  </si>
+  <si>
+    <t>fieldPhone</t>
+  </si>
+  <si>
+    <t>fieldAccountId</t>
+  </si>
+  <si>
+    <t>fieldSalutation</t>
+  </si>
+  <si>
+    <t>fieldFirstName</t>
+  </si>
+  <si>
+    <t>fieldLastName</t>
+  </si>
+  <si>
+    <t>fieldEmail</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -148,12 +145,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="5"/>
-      <color rgb="FF222222"/>
-      <name val="Consolas"/>
-      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -177,7 +168,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -189,7 +180,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -471,11 +461,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D795F61-CC1F-4314-B1D8-0852B981BA18}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="23.06640625" customWidth="1"/>
-    <col min="2" max="2" width="21.46484375" customWidth="1"/>
+    <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="37.19921875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -492,134 +482,123 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>28</v>
+        <v>10</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C10" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" t="s">
-        <v>34</v>
+        <v>25</v>
+      </c>
+      <c r="C11">
+        <v>20171</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12">
-        <v>20171</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" t="s">
-        <v>23</v>
+        <v>26</v>
+      </c>
+      <c r="C12" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -716,13 +695,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
         <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>